<commit_message>
v1.1.0 : trames Word refaites (cases à cocher, sections), classeurs Excel corrigés pour Excel en français
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/excel/registre-securite-vgp.xlsx
+++ b/excel/registre-securite-vgp.xlsx
@@ -20,10 +20,10 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="61">
   <si>
-    <t>Registre de sécurité · vérifications des appareils de levage</t>
+    <t xml:space="preserve">  Registre de sécurité · vérifications des appareils de levage</t>
   </si>
   <si>
-    <t>Une ligne par vérification : date, appareil, nature, vérificateur et rapport. Les observations et leurs suites se suivent dans le classeur « Suivi des réserves ».</t>
+    <t xml:space="preserve">  Une ligne par vérification : date, appareil, nature, vérificateur et rapport. Les observations et leurs suites se suivent dans le classeur « Suivi des réserves ».</t>
   </si>
   <si>
     <t>N°</t>
@@ -207,10 +207,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="&quot;Situation au &quot;dd/mm/yyyy"/>
+    <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -220,8 +221,8 @@
     </font>
     <font>
       <b/>
-      <color rgb="FF12314F"/>
-      <sz val="16"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="18"/>
     </font>
     <font>
       <i/>
@@ -234,6 +235,11 @@
     <font>
       <b/>
       <color rgb="FFFFFFFF"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF12314F"/>
+      <sz val="16"/>
     </font>
     <font>
       <b/>
@@ -259,7 +265,7 @@
       <color rgb="FF12805F"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -269,6 +275,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF12314F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF3F7FB"/>
       </patternFill>
     </fill>
     <fill>
@@ -314,51 +325,61 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -768,6 +789,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
+    <tabColor rgb="FF12314F"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:O304"/>
@@ -787,7 +809,7 @@
     <col min="14" max="15" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" ht="36" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -806,7 +828,7 @@
       <c r="N1" s="1"/>
       <c r="O1" s="1"/>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" ht="22" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -825,10 +847,14 @@
       <c r="N2" s="2"/>
       <c r="O2" s="2"/>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
-        <f>"Situation au "&amp;TEXT(TODAY(),"dd/mm/yyyy")</f>
-      </c>
+        <f>TODAY()</f>
+      </c>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
@@ -7179,9 +7205,10 @@
     </row>
   </sheetData>
   <autoFilter ref="A4:O304"/>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:O2"/>
+    <mergeCell ref="A3:E3"/>
   </mergeCells>
   <conditionalFormatting sqref="O5:O304">
     <cfRule type="expression" dxfId="0" priority="1">
@@ -7227,6 +7254,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <tabColor rgb="FF12805F"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:B10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
@@ -7235,63 +7266,63 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="9" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" s="3">
-        <f>"Situation au "&amp;TEXT(TODAY(),"dd/mm/yyyy")</f>
+      <c r="A2" s="10">
+        <f>TODAY()</f>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="9" t="s">
+      <c r="A4" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="B4" s="10">
+      <c r="B4" s="12">
         <f>COUNT('Registre'!$B$5:$B$304)</f>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="9" t="s">
+      <c r="A5" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="B5" s="11">
+      <c r="B5" s="13">
         <f>COUNTIF('Registre'!$O$5:$O$304,"Annexer le rapport")</f>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="9" t="s">
+      <c r="A6" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="B6" s="11">
+      <c r="B6" s="13">
         <f>COUNTIF('Registre'!$O$5:$O$304,"Suites à décider")</f>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="9" t="s">
+      <c r="A7" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="B7" s="12">
+      <c r="B7" s="14">
         <f>COUNTIF('Registre'!$O$5:$O$304,"Complet")</f>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="9" t="s">
+      <c r="A8" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="B8" s="13">
+      <c r="B8" s="15">
         <f>IF(COUNT('Registre'!$B$5:$B$304)=0,"Aucune",MAX('Registre'!$B$5:$B$304))</f>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A10" s="14" t="s">
+      <c r="A10" s="16" t="s">
         <v>23</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
   <headerFooter>
     <oddFooter>&amp;Lmodele-vgp.fr&amp;RPage &amp;P / &amp;N</oddFooter>
   </headerFooter>
@@ -7301,6 +7332,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
+    <tabColor rgb="FF9FB0C4"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:O304"/>
@@ -7320,7 +7352,7 @@
     <col min="14" max="15" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" ht="36" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -7339,7 +7371,7 @@
       <c r="N1" s="1"/>
       <c r="O1" s="1"/>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" ht="22" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -7358,10 +7390,14 @@
       <c r="N2" s="2"/>
       <c r="O2" s="2"/>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
-        <f>"Situation au "&amp;TEXT(TODAY(),"dd/mm/yyyy")</f>
-      </c>
+        <f>TODAY()</f>
+      </c>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
@@ -13784,9 +13820,10 @@
     </row>
   </sheetData>
   <autoFilter ref="A4:O304"/>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:O2"/>
+    <mergeCell ref="A3:E3"/>
   </mergeCells>
   <conditionalFormatting sqref="O5:O304">
     <cfRule type="expression" dxfId="3" priority="1">
@@ -13832,6 +13869,10 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <tabColor rgb="FF12805F"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:A17"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
@@ -13839,87 +13880,87 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="17" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="18" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" s="16" t="s">
+      <c r="A3" s="18" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" s="16" t="s">
+      <c r="A4" s="18" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" s="16" t="s">
+      <c r="A5" s="18" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" s="16" t="s">
+      <c r="A6" s="18" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" s="15" t="s">
+      <c r="A7" s="17" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8" s="16" t="s">
+      <c r="A8" s="18" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" s="16" t="s">
+      <c r="A9" s="18" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A10" s="17" t="s">
+      <c r="A10" s="19" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A11" s="16" t="s">
+      <c r="A11" s="18" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A12" s="15" t="s">
+      <c r="A12" s="17" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A13" s="16" t="s">
+      <c r="A13" s="18" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A14" s="17" t="s">
+      <c r="A14" s="19" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A15" s="16" t="s">
+      <c r="A15" s="18" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A16" s="16" t="s">
+      <c r="A16" s="18" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17" s="17" t="s">
+      <c r="A17" s="19" t="s">
         <v>60</v>
       </c>
     </row>
@@ -13930,6 +13971,9 @@
     <hyperlink ref="A17" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
+  <headerFooter>
+    <oddFooter>&amp;Lmodele-vgp.fr&amp;RPage &amp;P / &amp;N</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>